<commit_message>
chore: hosts.yml만 추적하도록 gitignore 설정
</commit_message>
<xml_diff>
--- a/firewall.xlsx
+++ b/firewall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\errop\aws_inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E7C3F24-9AB3-4B4D-ACB3-8DB090668D8B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5696A4-0CAD-450B-A913-EF3C54FF060A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7930" xr2:uid="{062FBF7F-E507-4C39-941B-5A744C0083F2}"/>
   </bookViews>
@@ -435,7 +435,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>22</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="4" spans="1:3">

</xml_diff>